<commit_message>
Improve character creation rules and localization
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/__tables__.xlsx
+++ b/Configs/GameConfig/Datas/__tables__.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R30f70c69fc5c4c7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3c43c37a1e9e45b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -957,6 +957,35 @@
       <x:c r="J24"/>
       <x:c r="K24"/>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25" t="str">
+        <x:v>dnd.TbTextLocalize</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>TextLocalize</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>TbTextLocalize@dnd_rule_content_luban_template.xlsx</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>text_key</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>c,s</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>DnD text localization table</x:v>
+      </x:c>
+      <x:c r="J25"/>
+      <x:c r="K25"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>